<commit_message>
feat(mame): bundle a resequencing sample run for steps 2.3 to 4
Load Sample Data now loads an independent resequencing run of the sample
plate, generated by the real pipeline (generate_mame_resequence_samples.py),
next to the original run. The writable workbooks and pick lists are copied
into <project>/sample_data/mame/{original,resequence}/ so step 2.4 manual
confirmation never edits bundled resources, joined with the project folder's
own separator so the step 4 evidence panel matches on Windows. A step 4 form
left on an earlier sample workbook is moved to the original copy; a workbook
the user picked is kept. Adds the missing mixed_depth_factor_amplicon_scale
run quality translation.

Signed-off-by: gyuminlee-repo <gyuminlee-repo@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/src-tauri/samples/mame/13_mame_verdict.xlsx
+++ b/src-tauri/samples/mame/13_mame_verdict.xlsx
@@ -8234,10 +8234,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O22"/>
+  <dimension ref="A1:O24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="29" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
     <col width="9" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
@@ -9524,7 +9524,7 @@
     <row r="20">
       <c r="A20" s="10" t="inlineStr">
         <is>
-          <t>Recovery (재현율)</t>
+          <t>Success rate (PASS)</t>
         </is>
       </c>
       <c r="B20" s="10" t="inlineStr">
@@ -9549,7 +9549,7 @@
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>recovered_mutants</t>
+          <t>passed_mutants</t>
         </is>
       </c>
       <c r="B21" s="12" t="n">
@@ -9572,11 +9572,13 @@
     <row r="22">
       <c r="A22" s="10" t="inlineStr">
         <is>
-          <t>total_mutants</t>
-        </is>
-      </c>
-      <c r="B22" s="10" t="n">
-        <v>16</v>
+          <t>Reproduced (PASS+AMBIGUOUS)</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
       </c>
       <c r="C22" s="10" t="n"/>
       <c r="D22" s="10" t="n"/>
@@ -9591,6 +9593,52 @@
       <c r="M22" s="10" t="n"/>
       <c r="N22" s="10" t="n"/>
       <c r="O22" s="10" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>recovered_mutants</t>
+        </is>
+      </c>
+      <c r="B23" s="12" t="n">
+        <v>16</v>
+      </c>
+      <c r="C23" s="12" t="n"/>
+      <c r="D23" s="12" t="n"/>
+      <c r="E23" s="12" t="n"/>
+      <c r="F23" s="12" t="n"/>
+      <c r="G23" s="12" t="n"/>
+      <c r="H23" s="12" t="n"/>
+      <c r="I23" s="12" t="n"/>
+      <c r="J23" s="12" t="n"/>
+      <c r="K23" s="12" t="n"/>
+      <c r="L23" s="12" t="n"/>
+      <c r="M23" s="12" t="n"/>
+      <c r="N23" s="12" t="n"/>
+      <c r="O23" s="12" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>total_mutants</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="C24" s="10" t="n"/>
+      <c r="D24" s="10" t="n"/>
+      <c r="E24" s="10" t="n"/>
+      <c r="F24" s="10" t="n"/>
+      <c r="G24" s="10" t="n"/>
+      <c r="H24" s="10" t="n"/>
+      <c r="I24" s="10" t="n"/>
+      <c r="J24" s="10" t="n"/>
+      <c r="K24" s="10" t="n"/>
+      <c r="L24" s="10" t="n"/>
+      <c r="M24" s="10" t="n"/>
+      <c r="N24" s="10" t="n"/>
+      <c r="O24" s="10" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -10226,7 +10274,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -10251,7 +10299,11 @@
           <t>kuma_version</t>
         </is>
       </c>
-      <c r="B2" s="10" t="inlineStr"/>
+      <c r="B2" s="10" t="inlineStr">
+        <is>
+          <t>0.16.76</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
@@ -10261,17 +10313,173 @@
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
-          <t>2026-08-31T05:28:20Z</t>
+          <t>2026-01-01T00:00:00Z</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
+          <t>reference_file</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>reference.fasta</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>reference_length</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>720</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>reference_sha256</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>e8d734949c2b74ac68d9ecd5aa1016aa75d496d292b124db7d4993f2e5409449</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>coding_window</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>0-720</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>mode</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>amplicon</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>ingest_mode</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>barcode</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>min_read_count</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>max_consensus_n_fraction</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>min_file_size_kb</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>many_cutoff</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>mixed_confident_depth_factor</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>mixed_confident_read_count</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>verdict_classes</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>PASS, AMBIGUOUS, MIXED, FRAMESHIFT, MANY, LOWDEPTH, NO_CALL, WRONG_AA</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
           <t>ngs_run_meta</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B17" s="10" t="inlineStr">
         <is>
           <t>(not found, no MinKNOW run folder detected)</t>
         </is>

</xml_diff>